<commit_message>
cambios hechos hasta el día 25/04 por la mañana
</commit_message>
<xml_diff>
--- a/krm/static/files/import_users.xlsx
+++ b/krm/static/files/import_users.xlsx
@@ -1,20 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onedrive-global.kpmg.com/personal/nicolasfernandorodri_kpmg_es/Documents/Desktop/krm-kpmg/krm/static/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onedrive-global.kpmg.com/personal/nataliamonsalve_kpmg_es/Documents/Documents/Repositorios Git/dev-sidenor/krm/static/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C069EB8F-C2FF-4C26-BA59-34E3634C7410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2622076-F73F-4890-86DE-8442A42F0CFF}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{5E178528-482D-47C0-BFDD-316439BC41D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99469A3A-6309-4136-9507-7578D1B64BFB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F4F32161-54CA-4CF9-9704-52D82463E579}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F4F32161-54CA-4CF9-9704-52D82463E579}"/>
   </bookViews>
   <sheets>
-    <sheet name="USER IMPORT" sheetId="1" r:id="rId1"/>
+    <sheet name="Users" sheetId="1" r:id="rId1"/>
+    <sheet name="Available values" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="Valores_Language">'Available values'!$C$2:$C$3</definedName>
+    <definedName name="Valores_Mail">'Available values'!$A$2:$A$3</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -33,96 +38,75 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Alvarez Revuelta, Mario</author>
-  </authors>
-  <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{A5C30231-CB32-4205-9EA5-A34F262F197C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alvarez Revuelta, Mario:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Introducir acrónimos de Compañías separados por coma</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{4530A937-635C-4E7B-944B-809781111FC7}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alvarez Revuelta, Mario:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-ES o EN</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Last Name</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Welcome email (Y/N)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>Company</t>
   </si>
   <si>
-    <t>Notification language</t>
-  </si>
-  <si>
-    <t>Username</t>
+    <t>Email address (*)</t>
+  </si>
+  <si>
+    <t>First Name (*)</t>
+  </si>
+  <si>
+    <t>Last Name (*)</t>
+  </si>
+  <si>
+    <t>Password (*)</t>
+  </si>
+  <si>
+    <t>Welcome email
+Y - Yes 
+N - No</t>
+  </si>
+  <si>
+    <t>Username (*)</t>
+  </si>
+  <si>
+    <t>Value's legend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User - Welcome email </t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Y - Yes</t>
+  </si>
+  <si>
+    <t>N - No</t>
+  </si>
+  <si>
+    <t>User - Notification language</t>
+  </si>
+  <si>
+    <t>en</t>
+  </si>
+  <si>
+    <t>es</t>
+  </si>
+  <si>
+    <t>Notification language
+en - English
+es - Spanish</t>
+  </si>
+  <si>
+    <t>en - English</t>
+  </si>
+  <si>
+    <t>es - Spanish</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -137,19 +121,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -168,7 +139,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -176,15 +147,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -204,9 +204,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -244,7 +244,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -350,7 +350,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -492,59 +492,126 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{097A7BC6-DDC8-4F67-9C17-E3B6D860BEF2}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{097A7BC6-DDC8-4F67-9C17-E3B6D860BEF2}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.5703125" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" customWidth="1"/>
-    <col min="3" max="3" width="24.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" customWidth="1"/>
-    <col min="7" max="7" width="24.42578125" customWidth="1"/>
-    <col min="8" max="8" width="22.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.1796875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="19.7265625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="21.81640625" style="4" customWidth="1"/>
+    <col min="4" max="5" width="16.81640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.453125" style="4" customWidth="1"/>
+    <col min="8" max="8" width="24.453125" style="4" customWidth="1"/>
+    <col min="9" max="9" width="22.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="H1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="3"/>
     </row>
   </sheetData>
+  <dataValidations count="4">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Email address" prompt="Please enter a valid email address without spaces, including the '@' symbol and a domain extension (e.g., .com, .org)_x000a_" sqref="A1:A7 A9:A1048576" xr:uid="{6B1B2D26-3848-40CA-8BA6-7A34D417BF02}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F1048576" xr:uid="{CD913ECE-9237-4683-98AC-71F056326949}">
+      <formula1>Valores_Mail</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1:H1048576" xr:uid="{BE011589-2205-42CC-9FE8-D72075B20D29}">
+      <formula1>Valores_Language</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Email address" prompt="Please enter a valid email address without spaces or uppercase letters, including the '@' symbol and a valid domain extension (e.g., .com, .org, etc)_x000a_" sqref="A8" xr:uid="{8F1127A5-7B21-420B-A5AB-E7EE72BEDE1E}"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE042D46-58F1-4AEA-919A-DF2A13611B2E}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="21.1796875" style="6" customWidth="1"/>
+    <col min="3" max="4" width="18.54296875" style="6" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="v1YEL6ACRlEzrNr4twHbNVbJ/qepph9en1zppqKWWronAnnPGwhD+rNFez+9CqtWvvppGRFaIGt4J6XS/RouRQ==" saltValue="N2k5b169ygpcnhYQCsyW3w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>